<commit_message>
Screen review: short sheet adds eight correctly excluded examples, one per layer
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test/experiments/paper_screen_20261019/review_20261027/review_sheet_short.xlsx
+++ b/test/experiments/paper_screen_20261019/review_20261027/review_sheet_short.xlsx
@@ -10,6 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1 确认我的判断" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2 政策问题" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3 补回抽查5篇" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4 正确排除的例子" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1704,4 +1705,576 @@
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="60" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="30" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>筛选层</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>标题</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>相关 GSE</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>筛选器的理由</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>我的说明</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>原文摘录</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>全文（本地）</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>全文（PMC）</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>DOI</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>GEO 链接</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>你的结论</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>你的备注</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>1 无全文</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Genomic biomarkers and clinical outcomes of physical activity</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="n"/>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>PMC 和 PDF 都没取到全文</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>综述</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>（没有取到全文）</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>（无）</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="n"/>
+      <c r="J2" s="3" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1111/j.1749-6632.2011.06091.x</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="n"/>
+      <c r="L2" s="4" t="inlineStr"/>
+      <c r="M2" s="4" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>2 非运动主题</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Comparative network-based analysis of toll-like receptor agonist, L-pampo signaling pathways in immune and cancer cells.</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>GSE264131</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>标题和摘要里没有运动相关词</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>TLR 激动剂，与运动无关</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>【数据声明】The RNA-seq datasets are available at [https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSE264131]. The data generated and analyzed in this study is included in this published article and its Supplementary Figures: Figure S1: Cancer cell viability induced by L-pampo treatment and RNA expression of TLR genes in THP-1, SW620, and PC-3; Figure S2: DEGs and KEGG pathway enrichment analysis results; Figure S3: Identification of perturbed modules using WGCNA and KEGG pathway analysis for the detecte
+【运动设计】方法/结果里没找到运动分组或方案的句子</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>fulltext/05_39060412.md</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>https://pmc.ncbi.nlm.nih.gov/articles/PMC11282102/</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1038/s41598-024-67000-1</t>
+        </is>
+      </c>
+      <c r="K3" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSE264131</t>
+        </is>
+      </c>
+      <c r="L3" s="4" t="inlineStr"/>
+      <c r="M3" s="4" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>3 无运动分组</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>The Effect of Resistance Training on the Rehabilitation of Elderly Patients with Sarcopenia: A Meta-Analysis</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="n"/>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>摘要、方法、结果里找不到本文自己的运动分组或方案</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>随机对照试验荟萃分析</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>【数据声明】Not applicable.
+【运动设计】方法/结果里没找到运动分组或方案的句子</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>fulltext/13_36497565.md</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>https://pmc.ncbi.nlm.nih.gov/articles/PMC9739568/</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/ijerph192315491</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="n"/>
+      <c r="L4" s="4" t="inlineStr"/>
+      <c r="M4" s="4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>4 无自有数据</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>hTERT Gene Expression and Athlete's Heart: A Study in Middle-Aged Endurance Athletes.</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="n"/>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>正文没有任何数据库编号</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>qPCR 测 hTERT</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>【数据声明】The original contributions presented in this study are included in the article. Further inquiries can be directed to the corresponding authors.
+【运动设计】…hic parameters including LVEDD, LV mass, and wall thicknesses (p &lt; 0.05). hTERT gene expression was 2.06-fold higher in athletes compared to controls. Significant positive correlations were observed between hTERT expression and VO_2peak, LVM, LV wall thicknesses, and right ventricular parameters. Conclusions: These fin…
+【运动设计】…d at the Department of Cardiology, Çukurova University, involving 38 middle-aged male elite runners and 37 healthy male sedentary individuals. The athlete group consisted of individuals aged 40 years and older who engaged in regular recreational running and participated in half-marathons and marathons. All participants…</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>fulltext/16_41010049.md</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>https://pmc.ncbi.nlm.nih.gov/articles/PMC12470116/</t>
+        </is>
+      </c>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/genes16091104</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="n"/>
+      <c r="L5" s="4" t="inlineStr"/>
+      <c r="M5" s="4" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>4 无自有数据：重用公共 GSE</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Exercise-primed extracellular vesicles improve cell-matrix adhesion and chondrocyte health.</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>GSE144627</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>正文提到的 GSE 被判为引用：GSE144627</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>用的是别人的 GSE144627</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">【数据声明】The raw data that support the experimental findings are included in article supplementary material. Any additional information required to reanalyze the data reported in this work is available from the corresponding author upon request.
+【results】To assess the global EV miRNA response to acute aerobic exercise, we accessed and evaluated the raw small RNA-seq data (GSE144627) from all 10 participants in the study.
+【results】**Figure 1** Small RNA-seq revealed that an acute bout of aerobic exercise significantly changed 16 EV miRNAs that primarily targeted the cell-matrix adhesion process A, An electronic database search yielded a total of 332 studies, of which 1 study (GSE144627)^3 was finally included.
+【methods】We accessed the archived small RNA-seq data (GSE144627) collected from the serum in older adults before exercise, immediately after exercise, and after 3 hours of recovery^3.
+【运动设计】…irculating EVs and chondrocytes, the cells resident in articular cartilage. Using the archived small RNA-seq data of EV before and after aerobic exercise, microRNA regulatory network analysis based on network propagation inferred that circulating EVs activated by aerobic exercise perturb chondrocyte-matrix interactions…
+【运动设计】…q. We identified only one study that performed small RNA-seq on circulating EVs in our target population, older adults, before and after exercise^3. In that study, male participants (n = 10, mean age: 69.3 years old) completed an acute bout of aerobic exercise on </t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>fulltext/20_37333349.md</t>
+        </is>
+      </c>
+      <c r="I6" s="3" t="inlineStr">
+        <is>
+          <t>https://pmc.ncbi.nlm.nih.gov/articles/PMC10274961/</t>
+        </is>
+      </c>
+      <c r="J6" s="3" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.21203/rs.3.rs-2958821/v1</t>
+        </is>
+      </c>
+      <c r="K6" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSE144627</t>
+        </is>
+      </c>
+      <c r="L6" s="4" t="inlineStr"/>
+      <c r="M6" s="4" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>4 无自有数据：需索取</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Normalization of gene expression data revisited: the three viewpoints of the transcriptome in human skeletal muscle undergoing load-induced hypertrophy and why they matter</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="n"/>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>数据声明写“向作者索取”</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>原始数据因隐私不公开</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>【数据声明】The codes and the count data used in analysis during the current study are available from the corresponding author on request. The raw sequence data is not publicly available due to patient confidentiality.
+【运动设计】…RNA-seq data from human skeletal muscle undergoing exercise-training-induced growth. Briefly, 25 participants conducted 12 weeks of high-load resistance training. Muscle biopsy specimens were sampled from m. vastus lateralis before, after two weeks of training (week 2) and after the intervention (week 12), and were sub…
+【运动设计】… 12 weeks of high-load resistance training. Muscle biopsy specimens were sampled from m. vastus lateralis before, after two weeks of training (week 2) and after the intervention (week 12), and were subsequently analyzed using RNA-seq. Transcript counts were modeled as (1) per-library-size, (2) per-total-RNA, and (3) pe…</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>fulltext/24_35717158.md</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t>https://pmc.ncbi.nlm.nih.gov/articles/PMC9206305/</t>
+        </is>
+      </c>
+      <c r="J7" s="3" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1186/s12859-022-04791-y</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="n"/>
+      <c r="L7" s="4" t="inlineStr"/>
+      <c r="M7" s="4" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>41</v>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>7 无计数：只有差异表</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Transcriptomic analysis reveals the impact of concurrent, resistance, and endurance training on skeletal muscle</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>GSE137832</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>GSE137832（de_tables_only；rnaseq；Homo sapiens；文件:de_tables_only；分组:Concurrent=12,Resistance=12,Endurance=12）</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>只有三张差异表</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>【数据声明】The dataset (GSE137832) analyzed during this study is available in the Gene Expression Omnibus (GEO) repository, https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSE137832. All other data are within the paper and its supplementary information files.
+【introduction】To address these gaps, this study utilizes the public gene expression dataset GSE137832 to systematically compare the effects of CET, RES, and END on the skeletal muscle transcriptome in healthy males under controlled experimental conditions.
+【methods】Data were obtained from the Gene Expression Omnibus (GEO) public database, specifically dataset GSE137832.
+【运动设计】…sis further demonstrated a universal activation of ECM remodeling and an inhibition of translation initiation processes post-training. Weighted gene co-expression and protein-protein interaction network analyses pinpointed core genes associated with each modality, including COL1A1/COL1A2 for CET and END, and SPARC/ASPN…
+【运动设计】…cally dataset GSE137832. This original study enrolled 18 healthy male subjects, stratified by lean body mass and evenly assigned to one of three training groups: Concurrent Exercise Training (CET), Resistance Exercise Training (RES), or Endurance Exercise Training (END). Baseline demographic and anthropometric characte…</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>fulltext/41_41637404.md</t>
+        </is>
+      </c>
+      <c r="I8" s="3" t="inlineStr">
+        <is>
+          <t>https://pmc.ncbi.nlm.nih.gov/articles/PMC12871994/</t>
+        </is>
+      </c>
+      <c r="J8" s="3" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1371/journal.pone.0340309</t>
+        </is>
+      </c>
+      <c r="K8" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSE137832</t>
+        </is>
+      </c>
+      <c r="L8" s="4" t="inlineStr"/>
+      <c r="M8" s="4" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>46</v>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>8 分组：只有一组</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Exercise suppresses IP6K3 to modulate BCAA metabolism and ferroptosis in MASLD.</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>GSE297883</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>GSE48452（no_own_deposit:linked_to_other_paper；microarray；Homo sapiens）
+GSE297883（single_group；rnaseq；Mus musculus；文件:raw_tar）</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>单细胞，2 个样本</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>【数据声明】Processed single-cell RNA-seq data of this study was deposited in the Gene Expression Omnibus under accession codes GSE297883. To review GEO accession GSE297883, go to (https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSE297883) and enter token “clivqciqzzqxjkp” into the box.
+【methods】Publicly available liver transcriptomic datasets related to non-alcoholic steatohepatitis (NASH) and bariatric intervention were obtained from the Gene Expression Omnibus (GEO) database, including GSE89632 (NASH cohort) and GSE48452 (bariatric intervention cohort).
+【methods】The raw scRNA-seq data from our study were deposited in the Gene Expression Omnibus (GEO) database under accession number GSE297883.
+【methods】The dataset GSE189600 (normal human liver and NASH human liver) was downloaded from the GEO database.
+【results】To explore exercise-responsive genes involved in MASLD, we analyzed transcriptomic datasets from a bariatric intervention cohort (GSE48452) and a NASH cohort (GSE89632).
+【results】A Volcano plot showing differentially expressed genes in the bariatric intervention cohort (GSE48452);
+【运动设计】…s with MASLD as well as mice. The functional role of IP6K3 was assessed by either hepatocyte-specific Ip6k3 deletion or exercise intervention in mice. Single-cell RNA sequencing (scRNA-seq), IP6K3 overexpression and knockdown, liquid chromatography–tandem mass spectrometry, and co-immunoprecipitation were used to explo…
+【运动设计】…ously [37]. Exercise training was initiated after 8 weeks of</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>fulltext/46_42420830.md</t>
+        </is>
+      </c>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t>https://pmc.ncbi.nlm.nih.gov/articles/PMC13628866/</t>
+        </is>
+      </c>
+      <c r="J9" s="3" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1186/s11658-026-00981-1</t>
+        </is>
+      </c>
+      <c r="K9" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSE297883</t>
+        </is>
+      </c>
+      <c r="L9" s="4" t="inlineStr"/>
+      <c r="M9" s="4" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="L2:L9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"确实不能用,其实能用,看不出"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I3" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J3" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K3" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H4" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I4" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J4" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H5" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I5" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J5" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I6" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J6" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K6" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H7" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I7" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J7" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I8" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J8" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K8" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I9" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J9" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K9" r:id="rId26"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>